<commit_message>
Subida general: módulos Unisport y FutbolDataAcademy actualizados
- RedDePases.py: correcciones menores
- FiltroSub23.py, addAge.py, generacionExcelEurocopa2024.py: mejoras en filtros y generación de Excel
- crearResumenDatos.py: nuevas métricas derivadas
- Nuevos scripts ModuloTres: exploración, limpieza, estadísticas descriptivas, contextualización
- Archivos Excel e imágenes actualizados (boxplots, correlación, histogramas)
- CLAUDE.md: instrucciones del repositorio

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Unisport-FutbolDataAcademy/Unisport/ModuloTres/eurocopa_sub23.xlsx
+++ b/Unisport-FutbolDataAcademy/Unisport/ModuloTres/eurocopa_sub23.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="253">
   <si>
     <t>player</t>
   </si>
@@ -37,7 +37,7 @@
     <t>pases_totales</t>
   </si>
   <si>
-    <t>pases_completados</t>
+    <t>pases_fallados</t>
   </si>
   <si>
     <t>pases_clave</t>
@@ -1380,7 +1380,7 @@
         <v>16</v>
       </c>
       <c r="H2">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -1604,7 +1604,7 @@
         <v>27</v>
       </c>
       <c r="H3">
-        <v>78</v>
+        <v>4</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -1828,7 +1828,7 @@
         <v>12</v>
       </c>
       <c r="H4">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="I4">
         <v>1</v>
@@ -2052,7 +2052,7 @@
         <v>92</v>
       </c>
       <c r="H5">
-        <v>271</v>
+        <v>20</v>
       </c>
       <c r="I5">
         <v>1</v>
@@ -2276,7 +2276,7 @@
         <v>235</v>
       </c>
       <c r="H6">
-        <v>737</v>
+        <v>21</v>
       </c>
       <c r="I6">
         <v>1</v>
@@ -2500,7 +2500,7 @@
         <v>71</v>
       </c>
       <c r="H7">
-        <v>182</v>
+        <v>16</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -2724,7 +2724,7 @@
         <v>3</v>
       </c>
       <c r="H8">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I8">
         <v>1</v>
@@ -2948,7 +2948,7 @@
         <v>88</v>
       </c>
       <c r="H9">
-        <v>319</v>
+        <v>14</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -3172,7 +3172,7 @@
         <v>193</v>
       </c>
       <c r="H10">
-        <v>747</v>
+        <v>30</v>
       </c>
       <c r="I10">
         <v>7</v>
@@ -3396,7 +3396,7 @@
         <v>17</v>
       </c>
       <c r="H11">
-        <v>117</v>
+        <v>6</v>
       </c>
       <c r="I11">
         <v>2</v>
@@ -3620,7 +3620,7 @@
         <v>211</v>
       </c>
       <c r="H12">
-        <v>557</v>
+        <v>33</v>
       </c>
       <c r="I12">
         <v>0</v>
@@ -3844,7 +3844,7 @@
         <v>72</v>
       </c>
       <c r="H13">
-        <v>419</v>
+        <v>26</v>
       </c>
       <c r="I13">
         <v>2</v>
@@ -4068,7 +4068,7 @@
         <v>265</v>
       </c>
       <c r="H14">
-        <v>893</v>
+        <v>27</v>
       </c>
       <c r="I14">
         <v>10</v>
@@ -4292,7 +4292,7 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15">
         <v>0</v>
@@ -4516,7 +4516,7 @@
         <v>109</v>
       </c>
       <c r="H16">
-        <v>350</v>
+        <v>16</v>
       </c>
       <c r="I16">
         <v>0</v>
@@ -4740,7 +4740,7 @@
         <v>34</v>
       </c>
       <c r="H17">
-        <v>177</v>
+        <v>4</v>
       </c>
       <c r="I17">
         <v>4</v>
@@ -4964,7 +4964,7 @@
         <v>0</v>
       </c>
       <c r="H18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I18">
         <v>0</v>
@@ -5179,7 +5179,7 @@
         <v>210</v>
       </c>
       <c r="E19" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F19">
         <v>638</v>
@@ -5188,7 +5188,7 @@
         <v>270</v>
       </c>
       <c r="H19">
-        <v>1020</v>
+        <v>47</v>
       </c>
       <c r="I19">
         <v>8</v>
@@ -5412,7 +5412,7 @@
         <v>0</v>
       </c>
       <c r="H20">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I20">
         <v>0</v>
@@ -5636,7 +5636,7 @@
         <v>78</v>
       </c>
       <c r="H21">
-        <v>279</v>
+        <v>19</v>
       </c>
       <c r="I21">
         <v>1</v>
@@ -5851,7 +5851,7 @@
         <v>213</v>
       </c>
       <c r="E22" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F22">
         <v>407</v>
@@ -5860,7 +5860,7 @@
         <v>110</v>
       </c>
       <c r="H22">
-        <v>585</v>
+        <v>24</v>
       </c>
       <c r="I22">
         <v>3</v>
@@ -6084,7 +6084,7 @@
         <v>75</v>
       </c>
       <c r="H23">
-        <v>234</v>
+        <v>29</v>
       </c>
       <c r="I23">
         <v>3</v>
@@ -6308,7 +6308,7 @@
         <v>40</v>
       </c>
       <c r="H24">
-        <v>207</v>
+        <v>14</v>
       </c>
       <c r="I24">
         <v>2</v>
@@ -6532,7 +6532,7 @@
         <v>156</v>
       </c>
       <c r="H25">
-        <v>487</v>
+        <v>40</v>
       </c>
       <c r="I25">
         <v>5</v>
@@ -6756,7 +6756,7 @@
         <v>88</v>
       </c>
       <c r="H26">
-        <v>347</v>
+        <v>8</v>
       </c>
       <c r="I26">
         <v>3</v>
@@ -6980,7 +6980,7 @@
         <v>8</v>
       </c>
       <c r="H27">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="I27">
         <v>0</v>
@@ -7204,7 +7204,7 @@
         <v>89</v>
       </c>
       <c r="H28">
-        <v>369</v>
+        <v>28</v>
       </c>
       <c r="I28">
         <v>3</v>
@@ -7428,7 +7428,7 @@
         <v>189</v>
       </c>
       <c r="H29">
-        <v>713</v>
+        <v>20</v>
       </c>
       <c r="I29">
         <v>7</v>
@@ -7652,7 +7652,7 @@
         <v>127</v>
       </c>
       <c r="H30">
-        <v>466</v>
+        <v>24</v>
       </c>
       <c r="I30">
         <v>6</v>
@@ -7876,7 +7876,7 @@
         <v>72</v>
       </c>
       <c r="H31">
-        <v>446</v>
+        <v>17</v>
       </c>
       <c r="I31">
         <v>4</v>
@@ -8100,7 +8100,7 @@
         <v>119</v>
       </c>
       <c r="H32">
-        <v>451</v>
+        <v>18</v>
       </c>
       <c r="I32">
         <v>4</v>
@@ -8324,7 +8324,7 @@
         <v>123</v>
       </c>
       <c r="H33">
-        <v>276</v>
+        <v>56</v>
       </c>
       <c r="I33">
         <v>0</v>
@@ -8548,7 +8548,7 @@
         <v>149</v>
       </c>
       <c r="H34">
-        <v>455</v>
+        <v>16</v>
       </c>
       <c r="I34">
         <v>0</v>
@@ -8763,7 +8763,7 @@
         <v>198</v>
       </c>
       <c r="E35" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F35">
         <v>94</v>
@@ -8772,7 +8772,7 @@
         <v>1</v>
       </c>
       <c r="H35">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="I35">
         <v>0</v>
@@ -8987,7 +8987,7 @@
         <v>214</v>
       </c>
       <c r="E36" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F36">
         <v>314</v>
@@ -8996,7 +8996,7 @@
         <v>67</v>
       </c>
       <c r="H36">
-        <v>231</v>
+        <v>18</v>
       </c>
       <c r="I36">
         <v>1</v>
@@ -9220,7 +9220,7 @@
         <v>200</v>
       </c>
       <c r="H37">
-        <v>579</v>
+        <v>27</v>
       </c>
       <c r="I37">
         <v>2</v>
@@ -9444,7 +9444,7 @@
         <v>152</v>
       </c>
       <c r="H38">
-        <v>462</v>
+        <v>11</v>
       </c>
       <c r="I38">
         <v>2</v>
@@ -9668,7 +9668,7 @@
         <v>172</v>
       </c>
       <c r="H39">
-        <v>798</v>
+        <v>22</v>
       </c>
       <c r="I39">
         <v>5</v>
@@ -9892,7 +9892,7 @@
         <v>27</v>
       </c>
       <c r="H40">
-        <v>126</v>
+        <v>5</v>
       </c>
       <c r="I40">
         <v>1</v>
@@ -10116,7 +10116,7 @@
         <v>118</v>
       </c>
       <c r="H41">
-        <v>598</v>
+        <v>24</v>
       </c>
       <c r="I41">
         <v>8</v>
@@ -10340,7 +10340,7 @@
         <v>21</v>
       </c>
       <c r="H42">
-        <v>96</v>
+        <v>3</v>
       </c>
       <c r="I42">
         <v>2</v>
@@ -10555,7 +10555,7 @@
         <v>225</v>
       </c>
       <c r="E43" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F43">
         <v>182</v>
@@ -10564,7 +10564,7 @@
         <v>2</v>
       </c>
       <c r="H43">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I43">
         <v>0</v>
@@ -10788,7 +10788,7 @@
         <v>74</v>
       </c>
       <c r="H44">
-        <v>230</v>
+        <v>4</v>
       </c>
       <c r="I44">
         <v>0</v>
@@ -11012,7 +11012,7 @@
         <v>160</v>
       </c>
       <c r="H45">
-        <v>524</v>
+        <v>11</v>
       </c>
       <c r="I45">
         <v>0</v>
@@ -11236,7 +11236,7 @@
         <v>374</v>
       </c>
       <c r="H46">
-        <v>1444</v>
+        <v>57</v>
       </c>
       <c r="I46">
         <v>5</v>
@@ -11460,7 +11460,7 @@
         <v>50</v>
       </c>
       <c r="H47">
-        <v>275</v>
+        <v>6</v>
       </c>
       <c r="I47">
         <v>2</v>
@@ -11684,7 +11684,7 @@
         <v>110</v>
       </c>
       <c r="H48">
-        <v>505</v>
+        <v>17</v>
       </c>
       <c r="I48">
         <v>1</v>
@@ -11908,7 +11908,7 @@
         <v>9</v>
       </c>
       <c r="H49">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="I49">
         <v>0</v>
@@ -12132,7 +12132,7 @@
         <v>89</v>
       </c>
       <c r="H50">
-        <v>478</v>
+        <v>18</v>
       </c>
       <c r="I50">
         <v>8</v>
@@ -12356,7 +12356,7 @@
         <v>203</v>
       </c>
       <c r="H51">
-        <v>681</v>
+        <v>19</v>
       </c>
       <c r="I51">
         <v>4</v>
@@ -12580,7 +12580,7 @@
         <v>193</v>
       </c>
       <c r="H52">
-        <v>586</v>
+        <v>33</v>
       </c>
       <c r="I52">
         <v>8</v>
@@ -12804,7 +12804,7 @@
         <v>205</v>
       </c>
       <c r="H53">
-        <v>913</v>
+        <v>44</v>
       </c>
       <c r="I53">
         <v>14</v>
@@ -13028,7 +13028,7 @@
         <v>20</v>
       </c>
       <c r="H54">
-        <v>71</v>
+        <v>5</v>
       </c>
       <c r="I54">
         <v>0</v>
@@ -13252,7 +13252,7 @@
         <v>2</v>
       </c>
       <c r="H55">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="I55">
         <v>0</v>
@@ -13476,7 +13476,7 @@
         <v>12</v>
       </c>
       <c r="H56">
-        <v>69</v>
+        <v>5</v>
       </c>
       <c r="I56">
         <v>0</v>
@@ -13700,7 +13700,7 @@
         <v>9</v>
       </c>
       <c r="H57">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="I57">
         <v>0</v>
@@ -13924,7 +13924,7 @@
         <v>84</v>
       </c>
       <c r="H58">
-        <v>310</v>
+        <v>6</v>
       </c>
       <c r="I58">
         <v>3</v>
@@ -14138,6 +14138,9 @@
       <c r="D59" t="s">
         <v>234</v>
       </c>
+      <c r="E59" t="s">
+        <v>249</v>
+      </c>
       <c r="F59">
         <v>84</v>
       </c>
@@ -14145,7 +14148,7 @@
         <v>0</v>
       </c>
       <c r="H59">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I59">
         <v>0</v>
@@ -14369,7 +14372,7 @@
         <v>84</v>
       </c>
       <c r="H60">
-        <v>241</v>
+        <v>7</v>
       </c>
       <c r="I60">
         <v>1</v>
@@ -14583,6 +14586,9 @@
       <c r="D61" t="s">
         <v>235</v>
       </c>
+      <c r="E61" t="s">
+        <v>250</v>
+      </c>
       <c r="F61">
         <v>92</v>
       </c>
@@ -14590,7 +14596,7 @@
         <v>1</v>
       </c>
       <c r="H61">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I61">
         <v>0</v>
@@ -14814,7 +14820,7 @@
         <v>453</v>
       </c>
       <c r="H62">
-        <v>1310</v>
+        <v>30</v>
       </c>
       <c r="I62">
         <v>0</v>
@@ -15038,7 +15044,7 @@
         <v>148</v>
       </c>
       <c r="H63">
-        <v>448</v>
+        <v>17</v>
       </c>
       <c r="I63">
         <v>0</v>
@@ -15262,7 +15268,7 @@
         <v>3</v>
       </c>
       <c r="H64">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="I64">
         <v>0</v>
@@ -15486,7 +15492,7 @@
         <v>27</v>
       </c>
       <c r="H65">
-        <v>114</v>
+        <v>13</v>
       </c>
       <c r="I65">
         <v>1</v>
@@ -15710,7 +15716,7 @@
         <v>7</v>
       </c>
       <c r="H66">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="I66">
         <v>0</v>
@@ -15934,7 +15940,7 @@
         <v>9</v>
       </c>
       <c r="H67">
-        <v>44</v>
+        <v>3</v>
       </c>
       <c r="I67">
         <v>0</v>
@@ -16158,7 +16164,7 @@
         <v>42</v>
       </c>
       <c r="H68">
-        <v>117</v>
+        <v>11</v>
       </c>
       <c r="I68">
         <v>0</v>
@@ -16382,7 +16388,7 @@
         <v>16</v>
       </c>
       <c r="H69">
-        <v>52</v>
+        <v>5</v>
       </c>
       <c r="I69">
         <v>0</v>
@@ -16606,7 +16612,7 @@
         <v>80</v>
       </c>
       <c r="H70">
-        <v>259</v>
+        <v>32</v>
       </c>
       <c r="I70">
         <v>1</v>
@@ -16821,7 +16827,7 @@
         <v>238</v>
       </c>
       <c r="E71" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F71">
         <v>402</v>
@@ -16830,7 +16836,7 @@
         <v>15</v>
       </c>
       <c r="H71">
-        <v>110</v>
+        <v>6</v>
       </c>
       <c r="I71">
         <v>0</v>
@@ -17054,7 +17060,7 @@
         <v>52</v>
       </c>
       <c r="H72">
-        <v>201</v>
+        <v>17</v>
       </c>
       <c r="I72">
         <v>5</v>
@@ -17278,7 +17284,7 @@
         <v>92</v>
       </c>
       <c r="H73">
-        <v>272</v>
+        <v>24</v>
       </c>
       <c r="I73">
         <v>0</v>
@@ -17502,7 +17508,7 @@
         <v>221</v>
       </c>
       <c r="H74">
-        <v>933</v>
+        <v>41</v>
       </c>
       <c r="I74">
         <v>11</v>
@@ -17726,7 +17732,7 @@
         <v>101</v>
       </c>
       <c r="H75">
-        <v>350</v>
+        <v>29</v>
       </c>
       <c r="I75">
         <v>1</v>
@@ -17950,7 +17956,7 @@
         <v>230</v>
       </c>
       <c r="H76">
-        <v>774</v>
+        <v>27</v>
       </c>
       <c r="I76">
         <v>5</v>
@@ -18174,7 +18180,7 @@
         <v>104</v>
       </c>
       <c r="H77">
-        <v>305</v>
+        <v>16</v>
       </c>
       <c r="I77">
         <v>1</v>
@@ -18398,7 +18404,7 @@
         <v>365</v>
       </c>
       <c r="H78">
-        <v>1144</v>
+        <v>41</v>
       </c>
       <c r="I78">
         <v>3</v>
@@ -18622,7 +18628,7 @@
         <v>124</v>
       </c>
       <c r="H79">
-        <v>420</v>
+        <v>30</v>
       </c>
       <c r="I79">
         <v>1</v>
@@ -18846,7 +18852,7 @@
         <v>48</v>
       </c>
       <c r="H80">
-        <v>249</v>
+        <v>14</v>
       </c>
       <c r="I80">
         <v>1</v>
@@ -19060,6 +19066,9 @@
       <c r="D81" t="s">
         <v>234</v>
       </c>
+      <c r="E81" t="s">
+        <v>249</v>
+      </c>
       <c r="F81">
         <v>78</v>
       </c>
@@ -19067,7 +19076,7 @@
         <v>15</v>
       </c>
       <c r="H81">
-        <v>80</v>
+        <v>3</v>
       </c>
       <c r="I81">
         <v>0</v>
@@ -19291,7 +19300,7 @@
         <v>92</v>
       </c>
       <c r="H82">
-        <v>434</v>
+        <v>9</v>
       </c>
       <c r="I82">
         <v>9</v>
@@ -19515,7 +19524,7 @@
         <v>111</v>
       </c>
       <c r="H83">
-        <v>348</v>
+        <v>19</v>
       </c>
       <c r="I83">
         <v>0</v>
@@ -19739,7 +19748,7 @@
         <v>113</v>
       </c>
       <c r="H84">
-        <v>444</v>
+        <v>26</v>
       </c>
       <c r="I84">
         <v>5</v>
@@ -19963,7 +19972,7 @@
         <v>54</v>
       </c>
       <c r="H85">
-        <v>408</v>
+        <v>11</v>
       </c>
       <c r="I85">
         <v>3</v>
@@ -20187,7 +20196,7 @@
         <v>238</v>
       </c>
       <c r="H86">
-        <v>723</v>
+        <v>18</v>
       </c>
       <c r="I86">
         <v>2</v>
@@ -20402,7 +20411,7 @@
         <v>243</v>
       </c>
       <c r="E87" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F87">
         <v>96</v>
@@ -20411,7 +20420,7 @@
         <v>1</v>
       </c>
       <c r="H87">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I87">
         <v>0</v>
@@ -20635,7 +20644,7 @@
         <v>178</v>
       </c>
       <c r="H88">
-        <v>546</v>
+        <v>43</v>
       </c>
       <c r="I88">
         <v>1</v>
@@ -20859,7 +20868,7 @@
         <v>53</v>
       </c>
       <c r="H89">
-        <v>241</v>
+        <v>14</v>
       </c>
       <c r="I89">
         <v>3</v>
@@ -21074,7 +21083,7 @@
         <v>214</v>
       </c>
       <c r="E90" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F90">
         <v>320</v>
@@ -21083,7 +21092,7 @@
         <v>93</v>
       </c>
       <c r="H90">
-        <v>292</v>
+        <v>21</v>
       </c>
       <c r="I90">
         <v>1</v>
@@ -21307,7 +21316,7 @@
         <v>0</v>
       </c>
       <c r="H91">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I91">
         <v>0</v>
@@ -21531,7 +21540,7 @@
         <v>2</v>
       </c>
       <c r="H92">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="I92">
         <v>0</v>
@@ -21755,7 +21764,7 @@
         <v>85</v>
       </c>
       <c r="H93">
-        <v>284</v>
+        <v>12</v>
       </c>
       <c r="I93">
         <v>1</v>
@@ -21979,7 +21988,7 @@
         <v>365</v>
       </c>
       <c r="H94">
-        <v>1061</v>
+        <v>16</v>
       </c>
       <c r="I94">
         <v>1</v>
@@ -22203,7 +22212,7 @@
         <v>185</v>
       </c>
       <c r="H95">
-        <v>736</v>
+        <v>31</v>
       </c>
       <c r="I95">
         <v>9</v>
@@ -22427,7 +22436,7 @@
         <v>17</v>
       </c>
       <c r="H96">
-        <v>99</v>
+        <v>2</v>
       </c>
       <c r="I96">
         <v>2</v>
@@ -22641,6 +22650,9 @@
       <c r="D97" t="s">
         <v>235</v>
       </c>
+      <c r="E97" t="s">
+        <v>250</v>
+      </c>
       <c r="F97">
         <v>189</v>
       </c>
@@ -22648,7 +22660,7 @@
         <v>106</v>
       </c>
       <c r="H97">
-        <v>301</v>
+        <v>11</v>
       </c>
       <c r="I97">
         <v>1</v>
@@ -22872,7 +22884,7 @@
         <v>39</v>
       </c>
       <c r="H98">
-        <v>212</v>
+        <v>4</v>
       </c>
       <c r="I98">
         <v>0</v>
@@ -23096,7 +23108,7 @@
         <v>3</v>
       </c>
       <c r="H99">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="I99">
         <v>0</v>

</xml_diff>